<commit_message>
feat: update polling data up to 2026-08-31 across Taipei, New Taipei, and Taichung with newly verified polls
</commit_message>
<xml_diff>
--- a/sheets_import/clearpoll_database.xlsx
+++ b/sheets_import/clearpoll_database.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -833,6 +833,108 @@
       <c r="K8" t="inlineStr">
         <is>
           <t>https://news.tvbs.com.tw/</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>nt2026-005</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>ettoday</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>ETtoday</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>1213</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>online</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>li:39.3,su:37.3</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>li:34.0,su:32.0</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>https://www.ettoday.net/</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>nt2026-006</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>era</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>年代民調</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>1070</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>phone</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>3</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>li:32.2,su:37.8</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>li:25.0,su:32.0</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>30</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>https://www.eranews.com.tw/</t>
         </is>
       </c>
     </row>
@@ -847,7 +949,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1210,6 +1312,57 @@
       <c r="K7" t="inlineStr">
         <is>
           <t>https://cnews.com.tw/</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>tc2026-007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>asia-pacific</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>新台灣國策智庫（委趨勢民調執行）</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>1159</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>phone</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>chiang_k:42.8,ho:36.1</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>chiang_k:36.0,ho:30.0</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>21.1</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>http://www.braintrust.tw/</t>
         </is>
       </c>
     </row>
@@ -1750,7 +1903,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2011,6 +2164,57 @@
       <c r="K5" t="inlineStr">
         <is>
           <t>https://www.zmedia.com.tw/</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>tp2026-005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>tpoc</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>TPOC台灣議題研究中心</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>1099</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>phone</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>2.96</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>chiang:48.4,shen:33.0</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>chiang:42.0,shen:26.0</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>18.6</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>https://www.tpoc.com.tw/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add early September polls (Beacon, TVBS) and implement AI Model election assessment briefs across all cities
</commit_message>
<xml_diff>
--- a/sheets_import/clearpoll_database.xlsx
+++ b/sheets_import/clearpoll_database.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -935,6 +935,108 @@
       <c r="K10" t="inlineStr">
         <is>
           <t>https://www.eranews.com.tw/</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>nt2026-007</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>beacon</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>信民協會（戴立安規劃／畢肯執行）</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>1071</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>phone</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>3</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>su:35.2,li:34.7</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>su:30.0,li:29.0</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>30.1</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>https://www.cmmedia.com.tw/</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>nt2026-008</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>tvbs</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>TVBS</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>1224</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>phone</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>li:39.8,su:33.1</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>li:33.0,su:27.0</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>27.1</v>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>https://news.tvbs.com.tw/</t>
         </is>
       </c>
     </row>

</xml_diff>